<commit_message>
feat: import LinearSVC and update stop word list in intent classification notebook
</commit_message>
<xml_diff>
--- a/SCCU_tfidf_results.xlsx
+++ b/SCCU_tfidf_results.xlsx
@@ -4801,7 +4801,7 @@
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>card control</t>
+          <t>what card control</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
@@ -4813,7 +4813,7 @@
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>my profil detail</t>
+          <t>what my profil detail</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
@@ -4825,7 +4825,7 @@
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>rate</t>
+          <t>what rate</t>
         </is>
       </c>
       <c r="B368" t="inlineStr">
@@ -4837,7 +4837,7 @@
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>travel plan</t>
+          <t>what travel plan</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
@@ -4849,7 +4849,7 @@
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>travel plan</t>
+          <t>what travel plan</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
@@ -4861,7 +4861,7 @@
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>your branch time</t>
+          <t>what your branch time</t>
         </is>
       </c>
       <c r="B371" t="inlineStr">
@@ -4873,7 +4873,7 @@
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>your current offer</t>
+          <t>what your current offer</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
@@ -4885,7 +4885,7 @@
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>do?</t>
+          <t>what do?</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
@@ -4897,7 +4897,7 @@
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>card control there</t>
+          <t>what card control there</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
@@ -4909,7 +4909,7 @@
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>card control</t>
+          <t>what card control</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
@@ -4921,7 +4921,7 @@
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>bill pay</t>
+          <t>what bill pay</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
@@ -4933,7 +4933,7 @@
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>my account statement</t>
+          <t>what my account statement</t>
         </is>
       </c>
       <c r="B377" t="inlineStr">
@@ -4945,7 +4945,7 @@
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>rate</t>
+          <t>what rate</t>
         </is>
       </c>
       <c r="B378" t="inlineStr">
@@ -4957,7 +4957,7 @@
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>offer</t>
+          <t>what offer</t>
         </is>
       </c>
       <c r="B379" t="inlineStr">
@@ -4969,7 +4969,7 @@
     <row r="380">
       <c r="A380" t="inlineStr">
         <is>
-          <t>travel plan avail</t>
+          <t>what travel plan avail</t>
         </is>
       </c>
       <c r="B380" t="inlineStr">
@@ -4981,7 +4981,7 @@
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>travel plan there</t>
+          <t>what travel plan there</t>
         </is>
       </c>
       <c r="B381" t="inlineStr">
@@ -5227,7 +5227,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>card control</t>
+          <t>what card control</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -5499,7 +5499,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>your branch time</t>
+          <t>what your branch time</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -5788,7 +5788,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>do?</t>
+          <t>what do?</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -6485,7 +6485,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>bill pay</t>
+          <t>what bill pay</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -6655,7 +6655,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>travel plan there</t>
+          <t>what travel plan there</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -7352,7 +7352,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>rate</t>
+          <t>what rate</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -7386,7 +7386,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>card control there</t>
+          <t>what card control there</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -8746,7 +8746,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>travel plan avail</t>
+          <t>what travel plan avail</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -9256,7 +9256,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>my account statement</t>
+          <t>what my account statement</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -9273,7 +9273,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>my profil detail</t>
+          <t>what my profil detail</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -9562,7 +9562,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>your current offer</t>
+          <t>what your current offer</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -10225,7 +10225,7 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>offer</t>
+          <t>what offer</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
@@ -10344,7 +10344,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>travel plan</t>
+          <t>what travel plan</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
@@ -10902,7 +10902,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>travel plan</t>
+          <t>what travel plan</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -11877,7 +11877,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>rate</t>
+          <t>what rate</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -12002,7 +12002,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>card control</t>
+          <t>what card control</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">

</xml_diff>